<commit_message>
Added Labour Innovation Persistence - currently set both employment persistence and unemployment persistence to 0%; - updated key function parameters; - improved input PL excel file structure (removed unused sheets) - added age guards for potential hourly earnings - changed MIN_HOURLY_WAGE_RATE from 0.0 to 1.5
</commit_message>
<xml_diff>
--- a/input/PL/parameters.xlsx
+++ b/input/PL/parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pineapple/IdeaProjects/SimPathsEU_JAN/input/PL/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pineapple/IdeaProjects/SimPathsEU_APR/input/PL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{468A27D1-6BDB-7E4F-92C4-2A4F66811887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D1881DF-B6E8-2D4D-919A-D17868ABF2C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24900" yWindow="2780" windowWidth="20300" windowHeight="19580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-22020" yWindow="4520" windowWidth="20300" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="1" r:id="rId1"/>
@@ -945,7 +945,7 @@
         <v>37</v>
       </c>
       <c r="B33" s="1">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
@@ -977,7 +977,7 @@
         <v>80</v>
       </c>
       <c r="B37" s="10">
-        <v>276</v>
+        <v>287</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="16" x14ac:dyDescent="0.2">
@@ -985,7 +985,7 @@
         <v>81</v>
       </c>
       <c r="B38" s="10">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="16" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
- fixed age guard bug causing donor DB match breaking - added additional multirun scenarios to config
</commit_message>
<xml_diff>
--- a/input/PL/parameters.xlsx
+++ b/input/PL/parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pineapple/IdeaProjects/SimPathsEU_APR/input/PL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D1881DF-B6E8-2D4D-919A-D17868ABF2C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FA1DF77-E497-7B46-AFCC-8E3518BC62E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-22020" yWindow="4520" windowWidth="20300" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-22020" yWindow="3940" windowWidth="20300" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="1" r:id="rId1"/>
@@ -977,7 +977,7 @@
         <v>80</v>
       </c>
       <c r="B37" s="10">
-        <v>287</v>
+        <v>276</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="16" x14ac:dyDescent="0.2">
@@ -985,7 +985,7 @@
         <v>81</v>
       </c>
       <c r="B38" s="10">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="16" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
- fixed age guard bug causing donor DB match breaking - added additional multirun scenarios to config - optimized disability, retirement, inSchool, fertility to produce less variance over runs - fixed ordering of inSchool alignment and inSchool process - by default enable Population and Cohabitation alignments
</commit_message>
<xml_diff>
--- a/input/PL/parameters.xlsx
+++ b/input/PL/parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pineapple/IdeaProjects/SimPathsEU_APR/input/PL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FA1DF77-E497-7B46-AFCC-8E3518BC62E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE8817CC-DB37-6A4D-908C-98875C54EC44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-22020" yWindow="3940" windowWidth="20300" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -977,7 +977,7 @@
         <v>80</v>
       </c>
       <c r="B37" s="10">
-        <v>276</v>
+        <v>287</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="16" x14ac:dyDescent="0.2">
@@ -985,7 +985,7 @@
         <v>81</v>
       </c>
       <c r="B38" s="10">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="16" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Corrected MAX_START_YEAR in parameters.xlsx
</commit_message>
<xml_diff>
--- a/input/PL/parameters.xlsx
+++ b/input/PL/parameters.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pineapple/IdeaProjects/SimPathsEU_APR/input/PL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE8817CC-DB37-6A4D-908C-98875C54EC44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EC85DE7-66D8-F144-8C4C-BBDE8169FA12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-22020" yWindow="3940" windowWidth="20300" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -873,7 +873,7 @@
         <v>28</v>
       </c>
       <c r="B24" s="1">
-        <v>2020</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>